<commit_message>
Fix exam publish, add question types, and direct Excel import
Publish shows errors and auto-adjusts question count. Supports multiple choice, true/false, and yes/no. Excel upload imports questions in one step with flexible Option1-6 and Answer columns.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/question-import-template.xlsx
+++ b/assets/question-import-template.xlsx
@@ -397,29 +397,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Order</v>
       </c>
       <c r="B1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="C1" t="str">
         <v>Question</v>
       </c>
-      <c r="C1" t="str">
-        <v>OptionA</v>
-      </c>
       <c r="D1" t="str">
-        <v>OptionB</v>
+        <v>Option1</v>
       </c>
       <c r="E1" t="str">
-        <v>OptionC</v>
+        <v>Option2</v>
       </c>
       <c r="F1" t="str">
-        <v>OptionD</v>
+        <v>Option3</v>
       </c>
       <c r="G1" t="str">
-        <v>Correct</v>
+        <v>Option4</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Answer</v>
       </c>
     </row>
     <row r="2">
@@ -427,21 +430,24 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
+        <v>multiple_choice</v>
+      </c>
+      <c r="C2" t="str">
         <v>What is the primary role of a healthcare assistant?</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Diagnose patients</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Support patient care under supervision</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Prescribe medication</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Perform surgery</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>B</v>
       </c>
     </row>
@@ -450,27 +456,67 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Which action best supports infection control?</v>
+        <v>true_false</v>
       </c>
       <c r="C3" t="str">
-        <v>Reuse gloves between patients</v>
+        <v>Hand hygiene should be performed before and after patient contact.</v>
       </c>
       <c r="D3" t="str">
-        <v>Skip hand hygiene when busy</v>
+        <v>True</v>
       </c>
       <c r="E3" t="str">
-        <v>Follow hand hygiene and PPE protocols</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Store PPE in patient rooms only</v>
-      </c>
-      <c r="G3" t="str">
-        <v>C</v>
+        <v>False</v>
+      </c>
+      <c r="H3" t="str">
+        <v>True</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>yes_no</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Should you report safeguarding concerns to your supervisor?</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E4" t="str">
+        <v>No</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>multiple_choice</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Which document records care given to a patient?</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Shopping list</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Care plan or care notes</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Staff rota only</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>